<commit_message>
Guardar resultados y cambios de experimentos de incertidumbre
</commit_message>
<xml_diff>
--- a/tests/CWC_test.xlsx
+++ b/tests/CWC_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Shared drives\Doctorado\Repositorios\uncertainty-informed-decision-making\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2CA56D1-3A03-4133-9393-A9B93BA6B289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1F4EF7F-30DB-4BF0-86A0-8344AAED5BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F24D7121-59CB-449E-9C6F-2D6B2C8932A6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F24D7121-59CB-449E-9C6F-2D6B2C8932A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
   <si>
     <t>width</t>
   </si>
@@ -420,7 +420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CBD6DA-D360-4581-9F38-D0DD83B82E52}">
-  <dimension ref="A4:N16"/>
+  <dimension ref="A4:N33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="13" width="4.5703125" bestFit="1" customWidth="1"/>
@@ -973,9 +973,556 @@
         <v>0</v>
       </c>
     </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21">
+        <v>8</v>
+      </c>
+      <c r="D21">
+        <v>0.1</v>
+      </c>
+      <c r="E21">
+        <v>0.2</v>
+      </c>
+      <c r="F21">
+        <v>0.3</v>
+      </c>
+      <c r="G21">
+        <v>0.4</v>
+      </c>
+      <c r="H21">
+        <v>0.5</v>
+      </c>
+      <c r="I21">
+        <v>0.6</v>
+      </c>
+      <c r="J21">
+        <v>0.7</v>
+      </c>
+      <c r="K21">
+        <v>0.8</v>
+      </c>
+      <c r="L21">
+        <v>0.9</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
+      </c>
+      <c r="N21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B22">
+        <v>0.1</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22" s="1">
+        <f>(1-$C22)*EXP(-$B$21*(MAX(0,(1-$B$22)-D$4)^2))</f>
+        <v>5.9760228950059375E-3</v>
+      </c>
+      <c r="E22" s="1">
+        <f t="shared" ref="E22:M32" si="5">(1-$C22)*EXP(-$B$21*(MAX(0,(1-$B$22)-E$4)^2))</f>
+        <v>1.9841094744370298E-2</v>
+      </c>
+      <c r="F22" s="1">
+        <f t="shared" si="5"/>
+        <v>5.6134762834133677E-2</v>
+      </c>
+      <c r="G22" s="1">
+        <f t="shared" si="5"/>
+        <v>0.1353352832366127</v>
+      </c>
+      <c r="H22" s="1">
+        <f t="shared" si="5"/>
+        <v>0.27803730045319408</v>
+      </c>
+      <c r="I22" s="1">
+        <f t="shared" si="5"/>
+        <v>0.48675225595997157</v>
+      </c>
+      <c r="J22" s="1">
+        <f t="shared" si="5"/>
+        <v>0.72614903707369072</v>
+      </c>
+      <c r="K22" s="1">
+        <f t="shared" si="5"/>
+        <v>0.92311634638663587</v>
+      </c>
+      <c r="L22" s="1">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="M22" s="1">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C23">
+        <v>0.1</v>
+      </c>
+      <c r="D23" s="1">
+        <f t="shared" ref="D23:D32" si="6">(1-$C23)*EXP(-$B$21*(MAX(0,(1-$B$22)-D$4)^2))</f>
+        <v>5.3784206055053439E-3</v>
+      </c>
+      <c r="E23" s="1">
+        <f t="shared" si="5"/>
+        <v>1.7856985269933269E-2</v>
+      </c>
+      <c r="F23" s="1">
+        <f t="shared" si="5"/>
+        <v>5.0521286550720308E-2</v>
+      </c>
+      <c r="G23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.12180175491295143</v>
+      </c>
+      <c r="H23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25023357040787469</v>
+      </c>
+      <c r="I23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.43807703036397444</v>
+      </c>
+      <c r="J23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.65353413336632171</v>
+      </c>
+      <c r="K23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.83080471174797232</v>
+      </c>
+      <c r="L23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.9</v>
+      </c>
+      <c r="M23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C24">
+        <v>0.2</v>
+      </c>
+      <c r="D24" s="1">
+        <f t="shared" si="6"/>
+        <v>4.7808183160047502E-3</v>
+      </c>
+      <c r="E24" s="1">
+        <f t="shared" si="5"/>
+        <v>1.587287579549624E-2</v>
+      </c>
+      <c r="F24" s="1">
+        <f t="shared" si="5"/>
+        <v>4.4907810267306947E-2</v>
+      </c>
+      <c r="G24" s="1">
+        <f t="shared" si="5"/>
+        <v>0.10826822658929017</v>
+      </c>
+      <c r="H24" s="1">
+        <f t="shared" si="5"/>
+        <v>0.22242984036255528</v>
+      </c>
+      <c r="I24" s="1">
+        <f t="shared" si="5"/>
+        <v>0.38940180476797726</v>
+      </c>
+      <c r="J24" s="1">
+        <f t="shared" si="5"/>
+        <v>0.5809192296589526</v>
+      </c>
+      <c r="K24" s="1">
+        <f t="shared" si="5"/>
+        <v>0.73849307710930878</v>
+      </c>
+      <c r="L24" s="1">
+        <f t="shared" si="5"/>
+        <v>0.8</v>
+      </c>
+      <c r="M24" s="1">
+        <f t="shared" si="5"/>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C25">
+        <v>0.3</v>
+      </c>
+      <c r="D25" s="1">
+        <f t="shared" si="6"/>
+        <v>4.1832160265041557E-3</v>
+      </c>
+      <c r="E25" s="1">
+        <f t="shared" si="5"/>
+        <v>1.3888766321059207E-2</v>
+      </c>
+      <c r="F25" s="1">
+        <f t="shared" si="5"/>
+        <v>3.9294333983893572E-2</v>
+      </c>
+      <c r="G25" s="1">
+        <f t="shared" si="5"/>
+        <v>9.4734698265628886E-2</v>
+      </c>
+      <c r="H25" s="1">
+        <f t="shared" si="5"/>
+        <v>0.19462611031723584</v>
+      </c>
+      <c r="I25" s="1">
+        <f t="shared" si="5"/>
+        <v>0.34072657917198007</v>
+      </c>
+      <c r="J25" s="1">
+        <f t="shared" si="5"/>
+        <v>0.50830432595158348</v>
+      </c>
+      <c r="K25" s="1">
+        <f t="shared" si="5"/>
+        <v>0.64618144247064502</v>
+      </c>
+      <c r="L25" s="1">
+        <f t="shared" si="5"/>
+        <v>0.7</v>
+      </c>
+      <c r="M25" s="1">
+        <f t="shared" si="5"/>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C26">
+        <v>0.4</v>
+      </c>
+      <c r="D26" s="1">
+        <f t="shared" si="6"/>
+        <v>3.5856137370035624E-3</v>
+      </c>
+      <c r="E26" s="1">
+        <f t="shared" si="5"/>
+        <v>1.1904656846622178E-2</v>
+      </c>
+      <c r="F26" s="1">
+        <f t="shared" si="5"/>
+        <v>3.3680857700480203E-2</v>
+      </c>
+      <c r="G26" s="1">
+        <f t="shared" si="5"/>
+        <v>8.1201169941967619E-2</v>
+      </c>
+      <c r="H26" s="1">
+        <f t="shared" si="5"/>
+        <v>0.16682238027191645</v>
+      </c>
+      <c r="I26" s="1">
+        <f t="shared" si="5"/>
+        <v>0.29205135357598294</v>
+      </c>
+      <c r="J26" s="1">
+        <f t="shared" si="5"/>
+        <v>0.43568942224421442</v>
+      </c>
+      <c r="K26" s="1">
+        <f t="shared" si="5"/>
+        <v>0.55386980783198148</v>
+      </c>
+      <c r="L26" s="1">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
+      <c r="M26" s="1">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C27">
+        <v>0.5</v>
+      </c>
+      <c r="D27" s="1">
+        <f t="shared" si="6"/>
+        <v>2.9880114475029688E-3</v>
+      </c>
+      <c r="E27" s="1">
+        <f t="shared" si="5"/>
+        <v>9.9205473721851491E-3</v>
+      </c>
+      <c r="F27" s="1">
+        <f t="shared" si="5"/>
+        <v>2.8067381417066838E-2</v>
+      </c>
+      <c r="G27" s="1">
+        <f t="shared" si="5"/>
+        <v>6.7667641618306351E-2</v>
+      </c>
+      <c r="H27" s="1">
+        <f t="shared" si="5"/>
+        <v>0.13901865022659704</v>
+      </c>
+      <c r="I27" s="1">
+        <f t="shared" si="5"/>
+        <v>0.24337612797998578</v>
+      </c>
+      <c r="J27" s="1">
+        <f t="shared" si="5"/>
+        <v>0.36307451853684536</v>
+      </c>
+      <c r="K27" s="1">
+        <f t="shared" si="5"/>
+        <v>0.46155817319331793</v>
+      </c>
+      <c r="L27" s="1">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="M27" s="1">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C28">
+        <v>0.6</v>
+      </c>
+      <c r="D28" s="1">
+        <f t="shared" si="6"/>
+        <v>2.3904091580023751E-3</v>
+      </c>
+      <c r="E28" s="1">
+        <f t="shared" si="5"/>
+        <v>7.9364378977481199E-3</v>
+      </c>
+      <c r="F28" s="1">
+        <f t="shared" si="5"/>
+        <v>2.2453905133653473E-2</v>
+      </c>
+      <c r="G28" s="1">
+        <f t="shared" si="5"/>
+        <v>5.4134113294645084E-2</v>
+      </c>
+      <c r="H28" s="1">
+        <f t="shared" si="5"/>
+        <v>0.11121492018127764</v>
+      </c>
+      <c r="I28" s="1">
+        <f t="shared" si="5"/>
+        <v>0.19470090238398863</v>
+      </c>
+      <c r="J28" s="1">
+        <f t="shared" si="5"/>
+        <v>0.2904596148294763</v>
+      </c>
+      <c r="K28" s="1">
+        <f t="shared" si="5"/>
+        <v>0.36924653855465439</v>
+      </c>
+      <c r="L28" s="1">
+        <f t="shared" si="5"/>
+        <v>0.4</v>
+      </c>
+      <c r="M28" s="1">
+        <f t="shared" si="5"/>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C29">
+        <v>0.7</v>
+      </c>
+      <c r="D29" s="1">
+        <f t="shared" si="6"/>
+        <v>1.7928068685017814E-3</v>
+      </c>
+      <c r="E29" s="1">
+        <f t="shared" si="5"/>
+        <v>5.95232842331109E-3</v>
+      </c>
+      <c r="F29" s="1">
+        <f t="shared" si="5"/>
+        <v>1.6840428850240105E-2</v>
+      </c>
+      <c r="G29" s="1">
+        <f t="shared" si="5"/>
+        <v>4.0600584970983816E-2</v>
+      </c>
+      <c r="H29" s="1">
+        <f t="shared" si="5"/>
+        <v>8.3411190135958241E-2</v>
+      </c>
+      <c r="I29" s="1">
+        <f t="shared" si="5"/>
+        <v>0.1460256767879915</v>
+      </c>
+      <c r="J29" s="1">
+        <f t="shared" si="5"/>
+        <v>0.21784471112210724</v>
+      </c>
+      <c r="K29" s="1">
+        <f t="shared" si="5"/>
+        <v>0.27693490391599079</v>
+      </c>
+      <c r="L29" s="1">
+        <f t="shared" si="5"/>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="M29" s="1">
+        <f t="shared" si="5"/>
+        <v>0.30000000000000004</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C30">
+        <v>0.8</v>
+      </c>
+      <c r="D30" s="1">
+        <f t="shared" si="6"/>
+        <v>1.1952045790011873E-3</v>
+      </c>
+      <c r="E30" s="1">
+        <f t="shared" si="5"/>
+        <v>3.9682189488740591E-3</v>
+      </c>
+      <c r="F30" s="1">
+        <f t="shared" si="5"/>
+        <v>1.1226952566826733E-2</v>
+      </c>
+      <c r="G30" s="1">
+        <f t="shared" si="5"/>
+        <v>2.7067056647322535E-2</v>
+      </c>
+      <c r="H30" s="1">
+        <f t="shared" si="5"/>
+        <v>5.5607460090638806E-2</v>
+      </c>
+      <c r="I30" s="1">
+        <f t="shared" si="5"/>
+        <v>9.7350451191994286E-2</v>
+      </c>
+      <c r="J30" s="1">
+        <f t="shared" si="5"/>
+        <v>0.14522980741473812</v>
+      </c>
+      <c r="K30" s="1">
+        <f t="shared" si="5"/>
+        <v>0.18462326927732714</v>
+      </c>
+      <c r="L30" s="1">
+        <f t="shared" si="5"/>
+        <v>0.19999999999999996</v>
+      </c>
+      <c r="M30" s="1">
+        <f t="shared" si="5"/>
+        <v>0.19999999999999996</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C31">
+        <v>0.9</v>
+      </c>
+      <c r="D31" s="1">
+        <f t="shared" si="6"/>
+        <v>5.9760228950059367E-4</v>
+      </c>
+      <c r="E31" s="1">
+        <f t="shared" si="5"/>
+        <v>1.9841094744370296E-3</v>
+      </c>
+      <c r="F31" s="1">
+        <f t="shared" si="5"/>
+        <v>5.6134762834133666E-3</v>
+      </c>
+      <c r="G31" s="1">
+        <f t="shared" si="5"/>
+        <v>1.3533528323661267E-2</v>
+      </c>
+      <c r="H31" s="1">
+        <f t="shared" si="5"/>
+        <v>2.7803730045319403E-2</v>
+      </c>
+      <c r="I31" s="1">
+        <f t="shared" si="5"/>
+        <v>4.8675225595997143E-2</v>
+      </c>
+      <c r="J31" s="1">
+        <f t="shared" si="5"/>
+        <v>7.2614903707369061E-2</v>
+      </c>
+      <c r="K31" s="1">
+        <f t="shared" si="5"/>
+        <v>9.231163463866357E-2</v>
+      </c>
+      <c r="L31" s="1">
+        <f t="shared" si="5"/>
+        <v>9.9999999999999978E-2</v>
+      </c>
+      <c r="M31" s="1">
+        <f t="shared" si="5"/>
+        <v>9.9999999999999978E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32" s="1">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="F32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="G32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="K32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="M32" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="D5:M5">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -987,7 +1534,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:M15">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D22:M32">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>